<commit_message>
registeration, login, currency, search by name works !!
</commit_message>
<xml_diff>
--- a/testdata/testdata.xlsx
+++ b/testdata/testdata.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/47784ea9286de5db/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="8_{29087799-15DF-4A11-88BF-E381255A6C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74F1E636-21F4-4259-A921-EEC1618625C4}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="8_{29087799-15DF-4A11-88BF-E381255A6C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE21595D-B24B-421A-8953-7DFD370E434B}"/>
   <bookViews>
-    <workbookView xWindow="1440" yWindow="2810" windowWidth="14400" windowHeight="7270" xr2:uid="{7B89C8A6-D0D8-4203-B56E-5109A7BE8483}"/>
+    <workbookView xWindow="3410" yWindow="3030" windowWidth="14400" windowHeight="7270" activeTab="1" xr2:uid="{7B89C8A6-D0D8-4203-B56E-5109A7BE8483}"/>
   </bookViews>
   <sheets>
     <sheet name="Register" sheetId="2" r:id="rId1"/>
-    <sheet name="Login" sheetId="1" r:id="rId2"/>
+    <sheet name="Login" sheetId="4" r:id="rId2"/>
     <sheet name="Search" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="35">
   <si>
     <t>email</t>
   </si>
@@ -41,60 +41,24 @@
     <t>expected_result</t>
   </si>
   <si>
-    <t>john.doe@example.com</t>
-  </si>
-  <si>
-    <t>jane.smith@example.com</t>
-  </si>
-  <si>
     <t>invalid@example.com</t>
   </si>
   <si>
     <t>nonexistent@example.com</t>
   </si>
   <si>
-    <t>valid@example.com</t>
-  </si>
-  <si>
-    <t>Password123</t>
-  </si>
-  <si>
-    <t>Test@456</t>
-  </si>
-  <si>
     <t>wrongpass</t>
   </si>
   <si>
     <t>anypass123</t>
   </si>
   <si>
-    <t>wrongpassword</t>
-  </si>
-  <si>
     <t>valid</t>
   </si>
   <si>
     <t>invalid</t>
   </si>
   <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>valid login- existing user</t>
-  </si>
-  <si>
-    <t>valid login - another existing user</t>
-  </si>
-  <si>
-    <t>invalid login - wrong password</t>
-  </si>
-  <si>
-    <t>invalid login - email doesn't exist</t>
-  </si>
-  <si>
-    <t>invalid login - existing email with wrong password</t>
-  </si>
-  <si>
     <t>first_name</t>
   </si>
   <si>
@@ -165,6 +129,12 @@
   </si>
   <si>
     <t>test@test.com</t>
+  </si>
+  <si>
+    <t>demo</t>
+  </si>
+  <si>
+    <t>demoaya@tutorialsninja.com</t>
   </si>
 </sst>
 </file>
@@ -188,18 +158,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -215,13 +179,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -542,16 +502,16 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="E1" t="s">
         <v>1</v>
@@ -560,85 +520,85 @@
         <v>2</v>
       </c>
       <c r="G1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>43</v>
+        <v>30</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>31</v>
       </c>
       <c r="D2">
         <v>1234567890</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>25</v>
+      <c r="E2" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>44</v>
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="D3">
         <v>1234567890</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>25</v>
+      <c r="E3" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="G3" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>44</v>
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="D4">
         <v>1234567890</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>25</v>
+      <c r="E4" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="C5" s="1"/>
       <c r="D5">
         <v>1234567890</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>25</v>
+      <c r="E5" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="G5" t="s">
         <v>0</v>
@@ -646,42 +606,42 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>25</v>
+      <c r="E6" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="G6" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="D7">
         <v>1234567890</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>33</v>
+      <c r="E7" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="G7" t="s">
         <v>1</v>
@@ -706,161 +666,61 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ABC61A3-A491-413A-907A-BBB42D0F3024}">
-  <dimension ref="A1:E18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D131ACE1-E027-4C31-B288-0DD7E4BF3079}">
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="26.08984375" customWidth="1"/>
-    <col min="2" max="2" width="14.26953125" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" customWidth="1"/>
-    <col min="4" max="4" width="17.36328125" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="3"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>5</v>
-      </c>
       <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="2"/>
-      <c r="C7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-    </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{99E2FE58-DAC5-4702-958C-FB03259443BF}"/>
-    <hyperlink ref="A3:A6" r:id="rId2" display="john.doe@example.com" xr:uid="{27564ED0-0FB3-42A5-B455-3CE6AD4B1472}"/>
-    <hyperlink ref="A3" r:id="rId3" xr:uid="{51830B4C-960E-4F6A-9E5E-112F25867E3A}"/>
-    <hyperlink ref="A4" r:id="rId4" xr:uid="{5C60BBEC-2F07-435E-BB13-627D0104A9E4}"/>
-    <hyperlink ref="A5" r:id="rId5" xr:uid="{78C03D65-1B39-419B-9DC7-5B5DF6CD188B}"/>
-    <hyperlink ref="A6" r:id="rId6" xr:uid="{0D663CF6-3F91-4CCC-86B0-421FDF93BBAB}"/>
-    <hyperlink ref="B3" r:id="rId7" xr:uid="{E3D89BAD-3EE4-42C5-9AF3-AC82D19E5F1A}"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{5D7DF444-826D-42F6-989A-3642EB41E7F4}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{744051B4-E365-455E-ADFE-AB06718F96F8}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{4A8E3938-497A-40EA-BA3F-AD22E3E8F2D1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
 
@@ -871,34 +731,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
testdata with adcanced search
</commit_message>
<xml_diff>
--- a/testdata/testdata.xlsx
+++ b/testdata/testdata.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/47784ea9286de5db/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="88" documentId="8_{29087799-15DF-4A11-88BF-E381255A6C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE21595D-B24B-421A-8953-7DFD370E434B}"/>
+  <xr:revisionPtr revIDLastSave="89" documentId="8_{29087799-15DF-4A11-88BF-E381255A6C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7006EB1A-E184-4FD6-A060-29D216316634}"/>
   <bookViews>
-    <workbookView xWindow="3410" yWindow="3030" windowWidth="14400" windowHeight="7270" activeTab="1" xr2:uid="{7B89C8A6-D0D8-4203-B56E-5109A7BE8483}"/>
+    <workbookView xWindow="3410" yWindow="2810" windowWidth="14400" windowHeight="7270" firstSheet="2" activeTab="2" xr2:uid="{7B89C8A6-D0D8-4203-B56E-5109A7BE8483}"/>
   </bookViews>
   <sheets>
     <sheet name="Register" sheetId="2" r:id="rId1"/>
     <sheet name="Login" sheetId="4" r:id="rId2"/>
-    <sheet name="Search" sheetId="3" r:id="rId3"/>
+    <sheet name="AdvancedSearch" sheetId="5" r:id="rId3"/>
+    <sheet name="Search" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="48">
   <si>
     <t>email</t>
   </si>
@@ -135,6 +136,45 @@
   </si>
   <si>
     <t>demoaya@tutorialsninja.com</t>
+  </si>
+  <si>
+    <t>search_keyword</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>expected_product</t>
+  </si>
+  <si>
+    <t>expected_no_results_message</t>
+  </si>
+  <si>
+    <t>mac</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>Components</t>
+  </si>
+  <si>
+    <t>Laptops &amp; Notebooks</t>
+  </si>
+  <si>
+    <t>MacBook</t>
+  </si>
+  <si>
+    <t>Phones &amp; PDAs</t>
+  </si>
+  <si>
+    <t>Apple Cinema 30</t>
+  </si>
+  <si>
+    <t>no product</t>
+  </si>
+  <si>
+    <t>iphone</t>
   </si>
 </sst>
 </file>
@@ -179,9 +219,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -725,6 +768,78 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82097BB1-68E8-435E-8F5D-9FECE59844C3}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.54296875" customWidth="1"/>
+    <col min="2" max="2" width="18.36328125" customWidth="1"/>
+    <col min="3" max="3" width="17.26953125" customWidth="1"/>
+    <col min="4" max="4" width="26.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECAA46D0-776C-4116-8A5C-6B72A78A6804}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
final version without checkout
</commit_message>
<xml_diff>
--- a/testdata/testdata.xlsx
+++ b/testdata/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/47784ea9286de5db/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="89" documentId="8_{29087799-15DF-4A11-88BF-E381255A6C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7006EB1A-E184-4FD6-A060-29D216316634}"/>
+  <xr:revisionPtr revIDLastSave="96" documentId="8_{29087799-15DF-4A11-88BF-E381255A6C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BAEC9D6-4419-4524-B6CE-3A647099B8FF}"/>
   <bookViews>
-    <workbookView xWindow="3410" yWindow="2810" windowWidth="14400" windowHeight="7270" firstSheet="2" activeTab="2" xr2:uid="{7B89C8A6-D0D8-4203-B56E-5109A7BE8483}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="2" xr2:uid="{7B89C8A6-D0D8-4203-B56E-5109A7BE8483}"/>
   </bookViews>
   <sheets>
     <sheet name="Register" sheetId="2" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="43">
   <si>
     <t>email</t>
   </si>
@@ -150,31 +150,16 @@
     <t>expected_no_results_message</t>
   </si>
   <si>
-    <t>mac</t>
-  </si>
-  <si>
     <t>Apple</t>
   </si>
   <si>
     <t>Components</t>
   </si>
   <si>
-    <t>Laptops &amp; Notebooks</t>
-  </si>
-  <si>
-    <t>MacBook</t>
-  </si>
-  <si>
-    <t>Phones &amp; PDAs</t>
-  </si>
-  <si>
     <t>Apple Cinema 30</t>
   </si>
   <si>
     <t>no product</t>
-  </si>
-  <si>
-    <t>iphone</t>
   </si>
 </sst>
 </file>
@@ -769,7 +754,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82097BB1-68E8-435E-8F5D-9FECE59844C3}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.54296875" customWidth="1"/>
@@ -794,44 +779,16 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" t="s">
         <v>40</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>41</v>
       </c>
-      <c r="C2" t="s">
-        <v>45</v>
-      </c>
       <c r="D2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B3" t="s">
         <v>42</v>
-      </c>
-      <c r="C3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>